<commit_message>
kommentare in fast access added und veränderte scripts getestet
</commit_message>
<xml_diff>
--- a/tools/output/test_coverage_history.xlsx
+++ b/tools/output/test_coverage_history.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="410">
   <si>
     <t>Testlauf 1 - 2026-09-18 21:17:25</t>
   </si>
@@ -1215,6 +1215,33 @@
   </si>
   <si>
     <t>(3328/4663)</t>
+  </si>
+  <si>
+    <t>Testlauf 42 - 2026-10-09 22:15:22</t>
+  </si>
+  <si>
+    <t>(3403/6472)</t>
+  </si>
+  <si>
+    <t>Testlauf 43 - 2026-10-09 22:45:54</t>
+  </si>
+  <si>
+    <t>(1871/2862)</t>
+  </si>
+  <si>
+    <t>(7695/13005)</t>
+  </si>
+  <si>
+    <t>(3411/6472)</t>
+  </si>
+  <si>
+    <t>(800/928)</t>
+  </si>
+  <si>
+    <t>(3289/4663)</t>
+  </si>
+  <si>
+    <t>(1561/2685)</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J724"/>
+  <dimension ref="A1:J760"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.0140705108643" customWidth="1"/>
@@ -17314,6 +17341,804 @@
         <v>244</v>
       </c>
     </row>
+    <row r="728">
+      <c r="A728" s="0" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C729" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E729" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G729" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I729" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C730" s="0">
+        <v>0.82</v>
+      </c>
+      <c r="D730" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="E730" s="0">
+        <v>0.66</v>
+      </c>
+      <c r="F730" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="G730" s="0">
+        <v>0.59</v>
+      </c>
+      <c r="H730" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="I730" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="J730" s="0" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C731" s="0">
+        <v>1</v>
+      </c>
+      <c r="D731" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E731" s="0">
+        <v>1</v>
+      </c>
+      <c r="F731" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G731" s="0">
+        <v>1</v>
+      </c>
+      <c r="H731" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I731" s="0">
+        <v>1</v>
+      </c>
+      <c r="J731" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C732" s="0">
+        <v>1</v>
+      </c>
+      <c r="D732" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E732" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F732" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G732" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H732" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I732" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J732" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C733" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="D733" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="E733" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="F733" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="G733" s="0">
+        <v>0.39</v>
+      </c>
+      <c r="H733" s="0" t="s">
+        <v>389</v>
+      </c>
+      <c r="I733" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J733" s="0" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C734" s="0">
+        <v>1</v>
+      </c>
+      <c r="D734" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E734" s="0">
+        <v>1</v>
+      </c>
+      <c r="F734" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G734" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H734" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I734" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J734" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C735" s="0">
+        <v>0.98</v>
+      </c>
+      <c r="D735" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="E735" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F735" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="G735" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H735" s="0" t="s">
+        <v>370</v>
+      </c>
+      <c r="I735" s="0">
+        <v>0.58</v>
+      </c>
+      <c r="J735" s="0" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C736" s="0">
+        <v>1</v>
+      </c>
+      <c r="D736" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E736" s="0">
+        <v>1</v>
+      </c>
+      <c r="F736" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G736" s="0">
+        <v>1</v>
+      </c>
+      <c r="H736" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I736" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J736" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C737" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D737" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E737" s="0">
+        <v>0.81</v>
+      </c>
+      <c r="F737" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="G737" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="H737" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I737" s="0">
+        <v>0.66</v>
+      </c>
+      <c r="J737" s="0" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C738" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D738" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E738" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F738" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="G738" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H738" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="I738" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J738" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C739" s="0">
+        <v>1</v>
+      </c>
+      <c r="D739" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E739" s="0">
+        <v>1</v>
+      </c>
+      <c r="F739" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G739" s="0">
+        <v>1</v>
+      </c>
+      <c r="H739" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I739" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J739" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C740" s="0">
+        <v>1</v>
+      </c>
+      <c r="D740" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="E740" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="F740" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="G740" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H740" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I740" s="0">
+        <v>0.41</v>
+      </c>
+      <c r="J740" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C741" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D741" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E741" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F741" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="G741" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H741" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="I741" s="0">
+        <v>0.57</v>
+      </c>
+      <c r="J741" s="0" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C742" s="0">
+        <v>1</v>
+      </c>
+      <c r="D742" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="E742" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="F742" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="G742" s="0">
+        <v>0.32</v>
+      </c>
+      <c r="H742" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="I742" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="J742" s="0" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="0" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C747" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="E747" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="G747" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="I747" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C748" s="0">
+        <v>0.82</v>
+      </c>
+      <c r="D748" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="E748" s="0">
+        <v>0.65</v>
+      </c>
+      <c r="F748" s="0" t="s">
+        <v>404</v>
+      </c>
+      <c r="G748" s="0">
+        <v>0.59</v>
+      </c>
+      <c r="H748" s="0" t="s">
+        <v>405</v>
+      </c>
+      <c r="I748" s="0">
+        <v>0.53</v>
+      </c>
+      <c r="J748" s="0" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="C749" s="0">
+        <v>1</v>
+      </c>
+      <c r="D749" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E749" s="0">
+        <v>1</v>
+      </c>
+      <c r="F749" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G749" s="0">
+        <v>1</v>
+      </c>
+      <c r="H749" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="I749" s="0">
+        <v>1</v>
+      </c>
+      <c r="J749" s="0" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C750" s="0">
+        <v>1</v>
+      </c>
+      <c r="D750" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E750" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="F750" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="G750" s="0">
+        <v>0.84</v>
+      </c>
+      <c r="H750" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I750" s="0">
+        <v>0.77</v>
+      </c>
+      <c r="J750" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C751" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="D751" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="E751" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="F751" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="G751" s="0">
+        <v>0.39</v>
+      </c>
+      <c r="H751" s="0" t="s">
+        <v>389</v>
+      </c>
+      <c r="I751" s="0">
+        <v>0.37</v>
+      </c>
+      <c r="J751" s="0" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C752" s="0">
+        <v>1</v>
+      </c>
+      <c r="D752" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E752" s="0">
+        <v>1</v>
+      </c>
+      <c r="F752" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="G752" s="0">
+        <v>0.91</v>
+      </c>
+      <c r="H752" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="I752" s="0">
+        <v>0.76</v>
+      </c>
+      <c r="J752" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C753" s="0">
+        <v>0.98</v>
+      </c>
+      <c r="D753" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="E753" s="0">
+        <v>0.86</v>
+      </c>
+      <c r="F753" s="0" t="s">
+        <v>407</v>
+      </c>
+      <c r="G753" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="H753" s="0" t="s">
+        <v>408</v>
+      </c>
+      <c r="I753" s="0">
+        <v>0.58</v>
+      </c>
+      <c r="J753" s="0" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C754" s="0">
+        <v>1</v>
+      </c>
+      <c r="D754" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E754" s="0">
+        <v>1</v>
+      </c>
+      <c r="F754" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="G754" s="0">
+        <v>1</v>
+      </c>
+      <c r="H754" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I754" s="0">
+        <v>0.93</v>
+      </c>
+      <c r="J754" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C755" s="0">
+        <v>0.85</v>
+      </c>
+      <c r="D755" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="E755" s="0">
+        <v>0.81</v>
+      </c>
+      <c r="F755" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="G755" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="H755" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I755" s="0">
+        <v>0.67</v>
+      </c>
+      <c r="J755" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C756" s="0">
+        <v>0.97</v>
+      </c>
+      <c r="D756" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E756" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="F756" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="G756" s="0">
+        <v>0.83</v>
+      </c>
+      <c r="H756" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="I756" s="0">
+        <v>0.64</v>
+      </c>
+      <c r="J756" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C757" s="0">
+        <v>1</v>
+      </c>
+      <c r="D757" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E757" s="0">
+        <v>1</v>
+      </c>
+      <c r="F757" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="G757" s="0">
+        <v>1</v>
+      </c>
+      <c r="H757" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I757" s="0">
+        <v>0.71</v>
+      </c>
+      <c r="J757" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C758" s="0">
+        <v>1</v>
+      </c>
+      <c r="D758" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="E758" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="F758" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="G758" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H758" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I758" s="0">
+        <v>0.41</v>
+      </c>
+      <c r="J758" s="0" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C759" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="D759" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E759" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="F759" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="G759" s="0">
+        <v>0.72</v>
+      </c>
+      <c r="H759" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="I759" s="0">
+        <v>0.57</v>
+      </c>
+      <c r="J759" s="0" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C760" s="0">
+        <v>1</v>
+      </c>
+      <c r="D760" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="E760" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="F760" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="G760" s="0">
+        <v>0.32</v>
+      </c>
+      <c r="H760" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="I760" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="J760" s="0" t="s">
+        <v>244</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>